<commit_message>
corrected wrong sigma_crip value and intorduced history
</commit_message>
<xml_diff>
--- a/calculation_python/outputs/Results_final.xlsx
+++ b/calculation_python/outputs/Results_final.xlsx
@@ -9529,7 +9529,7 @@
         <v>-81.344481801271</v>
       </c>
       <c r="C123">
-        <v>95.39821916139468</v>
+        <v>394.8659066068382</v>
       </c>
       <c r="D123" s="3">
         <v>0.7818454474839299</v>
@@ -9548,7 +9548,7 @@
         <v>-26.76457855379006</v>
       </c>
       <c r="H123">
-        <v>95.39821916139468</v>
+        <v>394.8659066068382</v>
       </c>
       <c r="I123" s="2">
         <v>2.3762306828947644</v>
@@ -9599,7 +9599,7 @@
         <v>-90.83144995136678</v>
       </c>
       <c r="C124">
-        <v>95.39821916139468</v>
+        <v>394.8659066068382</v>
       </c>
       <c r="D124" s="3">
         <v>0.7001849338342101</v>
@@ -9618,7 +9618,7 @@
         <v>-29.88681694059249</v>
       </c>
       <c r="H124">
-        <v>95.39821916139468</v>
+        <v>394.8659066068382</v>
       </c>
       <c r="I124" s="2">
         <v>2.127988835367836</v>
@@ -9669,7 +9669,7 @@
         <v>-88.57206446197429</v>
       </c>
       <c r="C125">
-        <v>111.63528374528528</v>
+        <v>491.79</v>
       </c>
       <c r="D125" s="3">
         <v>0.840259544010158</v>
@@ -9688,7 +9688,7 @@
         <v>-29.142888354098826</v>
       </c>
       <c r="H125">
-        <v>111.63528374528528</v>
+        <v>491.79</v>
       </c>
       <c r="I125" s="2">
         <v>2.553745585975506</v>
@@ -9739,7 +9739,7 @@
         <v>-90.68922801370987</v>
       </c>
       <c r="C126">
-        <v>95.39821916139468</v>
+        <v>394.8659066068382</v>
       </c>
       <c r="D126" s="3">
         <v>0.7012829877066394</v>
@@ -9758,7 +9758,7 @@
         <v>-29.839581392495596</v>
       </c>
       <c r="H126">
-        <v>95.39821916139468</v>
+        <v>394.8659066068382</v>
       </c>
       <c r="I126" s="2">
         <v>2.1313574053776</v>
@@ -9809,7 +9809,7 @@
         <v>-88.15960863220425</v>
       </c>
       <c r="C127">
-        <v>111.63528374528528</v>
+        <v>491.79</v>
       </c>
       <c r="D127" s="3">
         <v>0.8441907087785133</v>
@@ -9828,7 +9828,7 @@
         <v>-29.007400114058935</v>
       </c>
       <c r="H127">
-        <v>111.63528374528528</v>
+        <v>491.79</v>
       </c>
       <c r="I127" s="2">
         <v>2.565673662728092</v>
@@ -9879,7 +9879,7 @@
         <v>-90.65860152566356</v>
       </c>
       <c r="C128">
-        <v>95.39821916139468</v>
+        <v>394.8659066068382</v>
       </c>
       <c r="D128" s="3">
         <v>0.701519896667054</v>
@@ -9898,7 +9898,7 @@
         <v>-29.829711182426287</v>
       </c>
       <c r="H128">
-        <v>95.39821916139468</v>
+        <v>394.8659066068382</v>
       </c>
       <c r="I128" s="2">
         <v>2.132062640007436</v>
@@ -9949,7 +9949,7 @@
         <v>-90.09982110235616</v>
       </c>
       <c r="C129">
-        <v>111.63528374528528</v>
+        <v>491.79</v>
       </c>
       <c r="D129" s="3">
         <v>0.8260118786729825</v>
@@ -9968,7 +9968,7 @@
         <v>-29.64581693302714</v>
       </c>
       <c r="H129">
-        <v>111.63528374528528</v>
+        <v>491.79</v>
       </c>
       <c r="I129" s="2">
         <v>2.5104223865709963</v>
@@ -10019,7 +10019,7 @@
         <v>-92.7554930184054</v>
       </c>
       <c r="C130">
-        <v>111.63528374528528</v>
+        <v>491.79</v>
       </c>
       <c r="D130" s="3">
         <v>0.8023624270110779</v>
@@ -10038,7 +10038,7 @@
         <v>-30.519560889416937</v>
       </c>
       <c r="H130">
-        <v>111.63528374528528</v>
+        <v>491.79</v>
       </c>
       <c r="I130" s="2">
         <v>2.4385515494970376</v>
@@ -10089,7 +10089,7 @@
         <v>-82.49919236890014</v>
       </c>
       <c r="C131">
-        <v>111.63528374528528</v>
+        <v>491.79</v>
       </c>
       <c r="D131" s="3">
         <v>0.9021121341899635</v>
@@ -10108,7 +10108,7 @@
         <v>-27.144811699627247</v>
       </c>
       <c r="H131">
-        <v>111.63528374528528</v>
+        <v>491.79</v>
       </c>
       <c r="I131" s="2">
         <v>2.741721818533699</v>

</xml_diff>

<commit_message>
new analysis 42 to 55
</commit_message>
<xml_diff>
--- a/calculation_python/outputs/Results_final.xlsx
+++ b/calculation_python/outputs/Results_final.xlsx
@@ -2586,13 +2586,13 @@
         </is>
       </c>
       <c r="B32">
-        <v>3.0</v>
+        <v>2.1</v>
       </c>
       <c r="C32">
-        <v>42.0</v>
+        <v>55.0</v>
       </c>
       <c r="D32">
-        <v>9.375</v>
+        <v>11.371794871794872</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -2662,13 +2662,13 @@
         </is>
       </c>
       <c r="B33">
-        <v>3.0</v>
+        <v>2.1</v>
       </c>
       <c r="C33">
-        <v>42.0</v>
+        <v>55.0</v>
       </c>
       <c r="D33">
-        <v>9.375</v>
+        <v>11.371794871794872</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -2814,13 +2814,13 @@
         </is>
       </c>
       <c r="B35">
-        <v>3.0</v>
+        <v>2.1</v>
       </c>
       <c r="C35">
-        <v>42.0</v>
+        <v>55.0</v>
       </c>
       <c r="D35">
-        <v>9.375</v>
+        <v>11.371794871794872</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -2966,13 +2966,13 @@
         </is>
       </c>
       <c r="B37">
-        <v>3.0</v>
+        <v>2.1</v>
       </c>
       <c r="C37">
-        <v>42.0</v>
+        <v>55.0</v>
       </c>
       <c r="D37">
-        <v>9.375</v>
+        <v>11.371794871794872</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -3680,7 +3680,7 @@
         </is>
       </c>
       <c r="B46" s="2">
-        <v>4.301193798345203</v>
+        <v>4.294539485208779</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -3693,7 +3693,7 @@
         </is>
       </c>
       <c r="E46" s="2">
-        <v>1.6866418540863786</v>
+        <v>1.6875157757509338</v>
       </c>
       <c r="F46" t="inlineStr">
         <is>
@@ -3758,7 +3758,7 @@
         </is>
       </c>
       <c r="B47" s="2">
-        <v>3.6884435402944864</v>
+        <v>3.6730805994301385</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -3771,7 +3771,7 @@
         </is>
       </c>
       <c r="E47" s="2">
-        <v>1.666944271312615</v>
+        <v>1.6670271369762553</v>
       </c>
       <c r="F47" t="inlineStr">
         <is>
@@ -3836,7 +3836,7 @@
         </is>
       </c>
       <c r="B48" s="2">
-        <v>4.087221177684532</v>
+        <v>4.070226023595548</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -3849,7 +3849,7 @@
         </is>
       </c>
       <c r="E48" s="2">
-        <v>1.668801238354483</v>
+        <v>1.6686408621969662</v>
       </c>
       <c r="F48" t="inlineStr">
         <is>
@@ -3914,7 +3914,7 @@
         </is>
       </c>
       <c r="B49" s="2">
-        <v>3.50902472089724</v>
+        <v>3.481713704492909</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
@@ -3927,7 +3927,7 @@
         </is>
       </c>
       <c r="E49" s="2">
-        <v>1.682038230315753</v>
+        <v>1.682659409012414</v>
       </c>
       <c r="F49" t="inlineStr">
         <is>
@@ -3992,7 +3992,7 @@
         </is>
       </c>
       <c r="B50" s="2">
-        <v>3.5787936692572915</v>
+        <v>3.5498401609169714</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
@@ -4005,7 +4005,7 @@
         </is>
       </c>
       <c r="E50" s="2">
-        <v>1.664771826019221</v>
+        <v>1.6647747740362473</v>
       </c>
       <c r="F50" t="inlineStr">
         <is>
@@ -4070,7 +4070,7 @@
         </is>
       </c>
       <c r="B51" s="2">
-        <v>3.6458482906838636</v>
+        <v>3.615547258111587</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
@@ -4083,7 +4083,7 @@
         </is>
       </c>
       <c r="E51" s="2">
-        <v>1.7008442665353598</v>
+        <v>1.701527513301477</v>
       </c>
       <c r="F51" t="inlineStr">
         <is>
@@ -4148,7 +4148,7 @@
         </is>
       </c>
       <c r="B52" s="2">
-        <v>3.5850535102744696</v>
+        <v>3.5600560013789138</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
@@ -4161,7 +4161,7 @@
         </is>
       </c>
       <c r="E52" s="2">
-        <v>1.6878088128813222</v>
+        <v>1.6874119836051793</v>
       </c>
       <c r="F52" t="inlineStr">
         <is>
@@ -4226,7 +4226,7 @@
         </is>
       </c>
       <c r="B53" s="2">
-        <v>3.5144124862500896</v>
+        <v>3.4938078534445367</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
@@ -4239,7 +4239,7 @@
         </is>
       </c>
       <c r="E53" s="2">
-        <v>1.662728037239743</v>
+        <v>1.6624609946202498</v>
       </c>
       <c r="F53" t="inlineStr">
         <is>
@@ -4304,7 +4304,7 @@
         </is>
       </c>
       <c r="B54" s="2">
-        <v>3.5561105643466604</v>
+        <v>3.5464433839054657</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
@@ -4317,7 +4317,7 @@
         </is>
       </c>
       <c r="E54" s="2">
-        <v>1.6838591053754521</v>
+        <v>1.6855293650739018</v>
       </c>
       <c r="F54" t="inlineStr">
         <is>
@@ -4382,7 +4382,7 @@
         </is>
       </c>
       <c r="B55" s="2">
-        <v>3.5238223405166313</v>
+        <v>3.514717127714317</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
@@ -4395,7 +4395,7 @@
         </is>
       </c>
       <c r="E55" s="2">
-        <v>1.679848181759231</v>
+        <v>1.681147935189644</v>
       </c>
       <c r="F55" t="inlineStr">
         <is>
@@ -4460,7 +4460,7 @@
         </is>
       </c>
       <c r="B56" s="2">
-        <v>3.545439754214814</v>
+        <v>3.528771171420777</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
@@ -4473,7 +4473,7 @@
         </is>
       </c>
       <c r="E56" s="2">
-        <v>1.6631099594680236</v>
+        <v>1.6630291587106383</v>
       </c>
       <c r="F56" t="inlineStr">
         <is>
@@ -4538,7 +4538,7 @@
         </is>
       </c>
       <c r="B57" s="2">
-        <v>3.601389464987986</v>
+        <v>3.576240524551117</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
@@ -4551,7 +4551,7 @@
         </is>
       </c>
       <c r="E57" s="2">
-        <v>1.6905206533009576</v>
+        <v>1.6897405122820959</v>
       </c>
       <c r="F57" t="inlineStr">
         <is>
@@ -4616,7 +4616,7 @@
         </is>
       </c>
       <c r="B58" s="2">
-        <v>3.6017499875404604</v>
+        <v>3.5776794780537804</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
@@ -4629,7 +4629,7 @@
         </is>
       </c>
       <c r="E58" s="2">
-        <v>1.6900645403658348</v>
+        <v>1.6893991188567163</v>
       </c>
       <c r="F58" t="inlineStr">
         <is>
@@ -4694,7 +4694,7 @@
         </is>
       </c>
       <c r="B59" s="2">
-        <v>3.557702519826236</v>
+        <v>3.5404254210684223</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
@@ -4707,7 +4707,7 @@
         </is>
       </c>
       <c r="E59" s="2">
-        <v>1.6632604604971726</v>
+        <v>1.6632024378091932</v>
       </c>
       <c r="F59" t="inlineStr">
         <is>
@@ -4772,7 +4772,7 @@
         </is>
       </c>
       <c r="B60" s="2">
-        <v>3.5324641602630034</v>
+        <v>3.523021702996304</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
@@ -4785,7 +4785,7 @@
         </is>
       </c>
       <c r="E60" s="2">
-        <v>1.680566670291719</v>
+        <v>1.6817959788422372</v>
       </c>
       <c r="F60" t="inlineStr">
         <is>
@@ -4850,7 +4850,7 @@
         </is>
       </c>
       <c r="B61" s="2">
-        <v>3.5268185038247015</v>
+        <v>3.5190275203731756</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
@@ -4863,7 +4863,7 @@
         </is>
       </c>
       <c r="E61" s="2">
-        <v>1.6799073366104882</v>
+        <v>1.6813713678724984</v>
       </c>
       <c r="F61" t="inlineStr">
         <is>
@@ -4928,7 +4928,7 @@
         </is>
       </c>
       <c r="B62" s="2">
-        <v>3.5657260704394136</v>
+        <v>3.5467756990901034</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
@@ -4941,7 +4941,7 @@
         </is>
       </c>
       <c r="E62" s="2">
-        <v>1.6633480952664266</v>
+        <v>1.663251695154944</v>
       </c>
       <c r="F62" t="inlineStr">
         <is>
@@ -5006,7 +5006,7 @@
         </is>
       </c>
       <c r="B63" s="2">
-        <v>3.6064671336536427</v>
+        <v>3.581402668130521</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
@@ -5019,7 +5019,7 @@
         </is>
       </c>
       <c r="E63" s="2">
-        <v>1.6908258584692966</v>
+        <v>1.690045449056631</v>
       </c>
       <c r="F63" t="inlineStr">
         <is>
@@ -5084,7 +5084,7 @@
         </is>
       </c>
       <c r="B64" s="2">
-        <v>3.589251349115322</v>
+        <v>3.5665198857137694</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
@@ -5097,7 +5097,7 @@
         </is>
       </c>
       <c r="E64" s="2">
-        <v>1.689074530032031</v>
+        <v>1.6883566372538423</v>
       </c>
       <c r="F64" t="inlineStr">
         <is>
@@ -5162,7 +5162,7 @@
         </is>
       </c>
       <c r="B65" s="2">
-        <v>3.5477912418576256</v>
+        <v>3.5328351193910956</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
@@ -5175,7 +5175,7 @@
         </is>
       </c>
       <c r="E65" s="2">
-        <v>1.663412003997066</v>
+        <v>1.6634680426904453</v>
       </c>
       <c r="F65" t="inlineStr">
         <is>
@@ -5240,7 +5240,7 @@
         </is>
       </c>
       <c r="B66" s="2">
-        <v>3.5285270180689863</v>
+        <v>3.519364335261394</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
@@ -5253,7 +5253,7 @@
         </is>
       </c>
       <c r="E66" s="2">
-        <v>1.6807004975317723</v>
+        <v>1.6817633909275413</v>
       </c>
       <c r="F66" t="inlineStr">
         <is>
@@ -5318,7 +5318,7 @@
         </is>
       </c>
       <c r="B67" s="2">
-        <v>3.515338309057187</v>
+        <v>3.5155936415104048</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
@@ -5331,7 +5331,7 @@
         </is>
       </c>
       <c r="E67" s="2">
-        <v>1.6812972475356378</v>
+        <v>1.6815367722666439</v>
       </c>
       <c r="F67" t="inlineStr">
         <is>
@@ -5396,7 +5396,7 @@
         </is>
       </c>
       <c r="B68" s="2">
-        <v>3.428695913682162</v>
+        <v>3.426995493140162</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
@@ -5409,7 +5409,7 @@
         </is>
       </c>
       <c r="E68" s="2">
-        <v>1.6593048859127169</v>
+        <v>1.659180123358753</v>
       </c>
       <c r="F68" t="inlineStr">
         <is>
@@ -5474,7 +5474,7 @@
         </is>
       </c>
       <c r="B69" s="2">
-        <v>3.4806321855624103</v>
+        <v>3.479551564164482</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
@@ -5487,7 +5487,7 @@
         </is>
       </c>
       <c r="E69" s="2">
-        <v>1.676310212597096</v>
+        <v>1.6763548332210474</v>
       </c>
       <c r="F69" t="inlineStr">
         <is>
@@ -5552,7 +5552,7 @@
         </is>
       </c>
       <c r="B70" s="2">
-        <v>3.4922040211381313</v>
+        <v>3.4930192748248414</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
@@ -5565,7 +5565,7 @@
         </is>
       </c>
       <c r="E70" s="2">
-        <v>1.6884565331625876</v>
+        <v>1.6885501194476966</v>
       </c>
       <c r="F70" t="inlineStr">
         <is>
@@ -5630,7 +5630,7 @@
         </is>
       </c>
       <c r="B71" s="2">
-        <v>3.4218748848991707</v>
+        <v>3.423815006785263</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
@@ -5643,7 +5643,7 @@
         </is>
       </c>
       <c r="E71" s="2">
-        <v>1.657138996173068</v>
+        <v>1.657175741031117</v>
       </c>
       <c r="F71" t="inlineStr">
         <is>
@@ -5708,7 +5708,7 @@
         </is>
       </c>
       <c r="B72" s="2">
-        <v>3.3599742690377066</v>
+        <v>3.359111702685511</v>
       </c>
       <c r="C72" t="inlineStr">
         <is>
@@ -5721,7 +5721,7 @@
         </is>
       </c>
       <c r="E72" s="2">
-        <v>1.668248113738772</v>
+        <v>1.6680857389537442</v>
       </c>
       <c r="F72" t="inlineStr">
         <is>
@@ -5786,7 +5786,7 @@
         </is>
       </c>
       <c r="B73" s="2">
-        <v>3.9733601755204173</v>
+        <v>3.9737339091955555</v>
       </c>
       <c r="C73" t="inlineStr">
         <is>
@@ -5799,7 +5799,7 @@
         </is>
       </c>
       <c r="E73" s="2">
-        <v>1.6594348650974322</v>
+        <v>1.65947628079372</v>
       </c>
       <c r="F73" t="inlineStr">
         <is>
@@ -5864,7 +5864,7 @@
         </is>
       </c>
       <c r="B74" s="2">
-        <v>3.599040372870471</v>
+        <v>3.599476716958905</v>
       </c>
       <c r="C74" t="inlineStr">
         <is>
@@ -5877,7 +5877,7 @@
         </is>
       </c>
       <c r="E74" s="2">
-        <v>1.6631543428806377</v>
+        <v>1.6631500871577718</v>
       </c>
       <c r="F74" t="inlineStr">
         <is>
@@ -5942,7 +5942,7 @@
         </is>
       </c>
       <c r="B75" s="2">
-        <v>4.252970286864102</v>
+        <v>4.2530161533825614</v>
       </c>
       <c r="C75" t="inlineStr">
         <is>
@@ -5955,7 +5955,7 @@
         </is>
       </c>
       <c r="E75" s="2">
-        <v>1.683873439720825</v>
+        <v>1.6838837155031787</v>
       </c>
       <c r="F75" t="inlineStr">
         <is>
@@ -6020,7 +6020,7 @@
         </is>
       </c>
       <c r="B76" s="2">
-        <v>5.155641862782214</v>
+        <v>5.233671030157329</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
@@ -6033,7 +6033,7 @@
         </is>
       </c>
       <c r="E76" s="2">
-        <v>16.22973607704384</v>
+        <v>16.49570322843346</v>
       </c>
       <c r="F76" t="inlineStr">
         <is>
@@ -6098,7 +6098,7 @@
         </is>
       </c>
       <c r="B77" s="2">
-        <v>5.681830060164767</v>
+        <v>5.7869196584909615</v>
       </c>
       <c r="C77" t="inlineStr">
         <is>
@@ -6111,7 +6111,7 @@
         </is>
       </c>
       <c r="E77" s="2">
-        <v>17.267021973370976</v>
+        <v>17.586069643532014</v>
       </c>
       <c r="F77" t="inlineStr">
         <is>
@@ -6176,7 +6176,7 @@
         </is>
       </c>
       <c r="B78" s="2">
-        <v>5.123680292171515</v>
+        <v>5.200107458665923</v>
       </c>
       <c r="C78" t="inlineStr">
         <is>
@@ -6189,7 +6189,7 @@
         </is>
       </c>
       <c r="E78" s="2">
-        <v>15.060566328026994</v>
+        <v>15.268142620286948</v>
       </c>
       <c r="F78" t="inlineStr">
         <is>
@@ -6254,7 +6254,7 @@
         </is>
       </c>
       <c r="B79" s="2">
-        <v>4.999497597655756</v>
+        <v>5.1257002351411485</v>
       </c>
       <c r="C79" t="inlineStr">
         <is>
@@ -6267,7 +6267,7 @@
         </is>
       </c>
       <c r="E79" s="2">
-        <v>15.14067553414747</v>
+        <v>15.51560719450454</v>
       </c>
       <c r="F79" t="inlineStr">
         <is>
@@ -6332,7 +6332,7 @@
         </is>
       </c>
       <c r="B80" s="2">
-        <v>4.824482059845684</v>
+        <v>4.9270893200272505</v>
       </c>
       <c r="C80" t="inlineStr">
         <is>
@@ -6345,7 +6345,7 @@
         </is>
       </c>
       <c r="E80" s="2">
-        <v>14.6610433515765</v>
+        <v>14.972671698033828</v>
       </c>
       <c r="F80" t="inlineStr">
         <is>
@@ -6410,7 +6410,7 @@
         </is>
       </c>
       <c r="B81" s="2">
-        <v>5.0027577864274875</v>
+        <v>5.129495179995125</v>
       </c>
       <c r="C81" t="inlineStr">
         <is>
@@ -6423,7 +6423,7 @@
         </is>
       </c>
       <c r="E81" s="2">
-        <v>15.259425993862761</v>
+        <v>15.653439291635081</v>
       </c>
       <c r="F81" t="inlineStr">
         <is>
@@ -6488,7 +6488,7 @@
         </is>
       </c>
       <c r="B82" s="2">
-        <v>4.959644723298203</v>
+        <v>4.984452209156346</v>
       </c>
       <c r="C82" t="inlineStr">
         <is>
@@ -6501,7 +6501,7 @@
         </is>
       </c>
       <c r="E82" s="2">
-        <v>15.055322020642087</v>
+        <v>15.118014966194307</v>
       </c>
       <c r="F82" t="inlineStr">
         <is>
@@ -6566,7 +6566,7 @@
         </is>
       </c>
       <c r="B83" s="2">
-        <v>4.992410060618923</v>
+        <v>5.032613512196029</v>
       </c>
       <c r="C83" t="inlineStr">
         <is>
@@ -6579,7 +6579,7 @@
         </is>
       </c>
       <c r="E83" s="2">
-        <v>15.175082095165552</v>
+        <v>15.297291503145384</v>
       </c>
       <c r="F83" t="inlineStr">
         <is>
@@ -6644,7 +6644,7 @@
         </is>
       </c>
       <c r="B84" s="2">
-        <v>4.960587161729972</v>
+        <v>4.986156778850298</v>
       </c>
       <c r="C84" t="inlineStr">
         <is>
@@ -6657,7 +6657,7 @@
         </is>
       </c>
       <c r="E84" s="2">
-        <v>15.092338217047025</v>
+        <v>15.182809600877297</v>
       </c>
       <c r="F84" t="inlineStr">
         <is>
@@ -6722,7 +6722,7 @@
         </is>
       </c>
       <c r="B85" s="2">
-        <v>5.04043403514291</v>
+        <v>5.165918136448703</v>
       </c>
       <c r="C85" t="inlineStr">
         <is>
@@ -6735,7 +6735,7 @@
         </is>
       </c>
       <c r="E85" s="2">
-        <v>15.326694707660463</v>
+        <v>15.71023989335279</v>
       </c>
       <c r="F85" t="inlineStr">
         <is>
@@ -6800,7 +6800,7 @@
         </is>
       </c>
       <c r="B86" s="2">
-        <v>4.976815501375589</v>
+        <v>5.101030712900475</v>
       </c>
       <c r="C86" t="inlineStr">
         <is>
@@ -6813,7 +6813,7 @@
         </is>
       </c>
       <c r="E86" s="2">
-        <v>15.125469043908433</v>
+        <v>15.503007655811183</v>
       </c>
       <c r="F86" t="inlineStr">
         <is>
@@ -6878,7 +6878,7 @@
         </is>
       </c>
       <c r="B87" s="2">
-        <v>5.039920146786564</v>
+        <v>5.165273269807008</v>
       </c>
       <c r="C87" t="inlineStr">
         <is>
@@ -6891,7 +6891,7 @@
         </is>
       </c>
       <c r="E87" s="2">
-        <v>15.30887531966145</v>
+        <v>15.687645560757037</v>
       </c>
       <c r="F87" t="inlineStr">
         <is>
@@ -6956,7 +6956,7 @@
         </is>
       </c>
       <c r="B88" s="2">
-        <v>4.9613652079741515</v>
+        <v>4.981449185250068</v>
       </c>
       <c r="C88" t="inlineStr">
         <is>
@@ -6969,7 +6969,7 @@
         </is>
       </c>
       <c r="E88" s="2">
-        <v>15.078164284063877</v>
+        <v>15.138962630409768</v>
       </c>
       <c r="F88" t="inlineStr">
         <is>
@@ -7034,7 +7034,7 @@
         </is>
       </c>
       <c r="B89" s="2">
-        <v>4.999061936104497</v>
+        <v>5.02728203485955</v>
       </c>
       <c r="C89" t="inlineStr">
         <is>
@@ -7047,7 +7047,7 @@
         </is>
       </c>
       <c r="E89" s="2">
-        <v>15.192716621206868</v>
+        <v>15.278506714153767</v>
       </c>
       <c r="F89" t="inlineStr">
         <is>
@@ -7112,7 +7112,7 @@
         </is>
       </c>
       <c r="B90" s="2">
-        <v>4.961365737700774</v>
+        <v>4.981475352561514</v>
       </c>
       <c r="C90" t="inlineStr">
         <is>
@@ -7125,7 +7125,7 @@
         </is>
       </c>
       <c r="E90" s="2">
-        <v>15.078509225468425</v>
+        <v>15.139891175907504</v>
       </c>
       <c r="F90" t="inlineStr">
         <is>
@@ -7190,7 +7190,7 @@
         </is>
       </c>
       <c r="B91" s="2">
-        <v>5.0447011658333745</v>
+        <v>5.16935707939105</v>
       </c>
       <c r="C91" t="inlineStr">
         <is>
@@ -7203,7 +7203,7 @@
         </is>
       </c>
       <c r="E91" s="2">
-        <v>15.32356990986941</v>
+        <v>15.699231617631261</v>
       </c>
       <c r="F91" t="inlineStr">
         <is>
@@ -7268,7 +7268,7 @@
         </is>
       </c>
       <c r="B92" s="2">
-        <v>5.001591445607465</v>
+        <v>5.122614445027513</v>
       </c>
       <c r="C92" t="inlineStr">
         <is>
@@ -7281,7 +7281,7 @@
         </is>
       </c>
       <c r="E92" s="2">
-        <v>15.200660998924192</v>
+        <v>15.568501633359912</v>
       </c>
       <c r="F92" t="inlineStr">
         <is>
@@ -7346,7 +7346,7 @@
         </is>
       </c>
       <c r="B93" s="2">
-        <v>5.045256018186837</v>
+        <v>5.170103630949604</v>
       </c>
       <c r="C93" t="inlineStr">
         <is>
@@ -7359,7 +7359,7 @@
         </is>
       </c>
       <c r="E93" s="2">
-        <v>15.341913598727217</v>
+        <v>15.724604615458013</v>
       </c>
       <c r="F93" t="inlineStr">
         <is>
@@ -7424,7 +7424,7 @@
         </is>
       </c>
       <c r="B94" s="2">
-        <v>4.964652748908433</v>
+        <v>4.97366834601145</v>
       </c>
       <c r="C94" t="inlineStr">
         <is>
@@ -7437,7 +7437,7 @@
         </is>
       </c>
       <c r="E94" s="2">
-        <v>15.079174688937757</v>
+        <v>15.089237191805108</v>
       </c>
       <c r="F94" t="inlineStr">
         <is>
@@ -7502,7 +7502,7 @@
         </is>
       </c>
       <c r="B95" s="2">
-        <v>4.9861599890550306</v>
+        <v>4.999293203769039</v>
       </c>
       <c r="C95" t="inlineStr">
         <is>
@@ -7515,7 +7515,7 @@
         </is>
       </c>
       <c r="E95" s="2">
-        <v>15.154250641894917</v>
+        <v>15.194179631312323</v>
       </c>
       <c r="F95" t="inlineStr">
         <is>
@@ -7580,7 +7580,7 @@
         </is>
       </c>
       <c r="B96" s="2">
-        <v>4.965279264361973</v>
+        <v>4.975335181877686</v>
       </c>
       <c r="C96" t="inlineStr">
         <is>
@@ -7593,7 +7593,7 @@
         </is>
       </c>
       <c r="E96" s="2">
-        <v>15.100411022038951</v>
+        <v>15.148426055178707</v>
       </c>
       <c r="F96" t="inlineStr">
         <is>
@@ -7658,7 +7658,7 @@
         </is>
       </c>
       <c r="B97" s="2">
-        <v>4.931794133701363</v>
+        <v>4.9307134860945006</v>
       </c>
       <c r="C97" t="inlineStr">
         <is>
@@ -7671,7 +7671,7 @@
         </is>
       </c>
       <c r="E97" s="2">
-        <v>15.035008784212707</v>
+        <v>15.028317925993223</v>
       </c>
       <c r="F97" t="inlineStr">
         <is>
@@ -7736,7 +7736,7 @@
         </is>
       </c>
       <c r="B98" s="2">
-        <v>4.7849141055644475</v>
+        <v>4.78489784595573</v>
       </c>
       <c r="C98" t="inlineStr">
         <is>
@@ -7749,7 +7749,7 @@
         </is>
       </c>
       <c r="E98" s="2">
-        <v>14.542721507637484</v>
+        <v>14.542670305074076</v>
       </c>
       <c r="F98" t="inlineStr">
         <is>
@@ -7814,7 +7814,7 @@
         </is>
       </c>
       <c r="B99" s="2">
-        <v>4.9290152363824795</v>
+        <v>4.928137542623586</v>
       </c>
       <c r="C99" t="inlineStr">
         <is>
@@ -7827,7 +7827,7 @@
         </is>
       </c>
       <c r="E99" s="2">
-        <v>14.93499130957703</v>
+        <v>14.935681370128268</v>
       </c>
       <c r="F99" t="inlineStr">
         <is>
@@ -7892,7 +7892,7 @@
         </is>
       </c>
       <c r="B100" s="2">
-        <v>5.234278255354964</v>
+        <v>5.23451175031139</v>
       </c>
       <c r="C100" t="inlineStr">
         <is>
@@ -7905,7 +7905,7 @@
         </is>
       </c>
       <c r="E100" s="2">
-        <v>15.399590811443295</v>
+        <v>15.404025749596126</v>
       </c>
       <c r="F100" t="inlineStr">
         <is>
@@ -7970,7 +7970,7 @@
         </is>
       </c>
       <c r="B101" s="2">
-        <v>5.775451501429353</v>
+        <v>5.776155777899696</v>
       </c>
       <c r="C101" t="inlineStr">
         <is>
@@ -7983,7 +7983,7 @@
         </is>
       </c>
       <c r="E101" s="2">
-        <v>17.553103165876326</v>
+        <v>17.555245132299873</v>
       </c>
       <c r="F101" t="inlineStr">
         <is>
@@ -8048,7 +8048,7 @@
         </is>
       </c>
       <c r="B102" s="2">
-        <v>5.265855361256913</v>
+        <v>5.2658482003530445</v>
       </c>
       <c r="C102" t="inlineStr">
         <is>
@@ -8061,7 +8061,7 @@
         </is>
       </c>
       <c r="E102" s="2">
-        <v>16.554103369707477</v>
+        <v>16.549725707429914</v>
       </c>
       <c r="F102" t="inlineStr">
         <is>
@@ -8536,22 +8536,22 @@
         </is>
       </c>
       <c r="B108">
-        <v>-59.20624287923199</v>
+        <v>-59.59139251708999</v>
       </c>
       <c r="C108">
-        <v>18.600112915039333</v>
+        <v>18.600114186605</v>
       </c>
       <c r="D108">
-        <v>30.77696355183933</v>
+        <v>30.770037333170666</v>
       </c>
       <c r="E108">
         <v>5.7844444444444445</v>
       </c>
       <c r="F108">
-        <v>5.271894605097841</v>
+        <v>5.26459119230698</v>
       </c>
       <c r="G108" s="2">
-        <v>2.060691368631207</v>
+        <v>2.046065081166741</v>
       </c>
       <c r="H108" t="inlineStr">
         <is>
@@ -8564,22 +8564,22 @@
         </is>
       </c>
       <c r="J108">
-        <v>-19.481197992960332</v>
+        <v>-19.607909838358665</v>
       </c>
       <c r="K108">
-        <v>6.120553016662667</v>
+        <v>6.120551109314</v>
       </c>
       <c r="L108">
-        <v>121.52023824055999</v>
+        <v>121.49289194742833</v>
       </c>
       <c r="M108">
         <v>5.7844444444444445</v>
       </c>
       <c r="N108">
-        <v>5.271964764870574</v>
+        <v>5.2646612879452235</v>
       </c>
       <c r="O108" s="2">
-        <v>1.208587315789261</v>
+        <v>1.2073604371471607</v>
       </c>
       <c r="P108" t="inlineStr">
         <is>
@@ -8594,22 +8594,22 @@
         </is>
       </c>
       <c r="B109">
-        <v>-72.87734222412134</v>
+        <v>-73.85754903157567</v>
       </c>
       <c r="C109">
         <v>18.600112915039002</v>
       </c>
       <c r="D109">
-        <v>30.547233581543</v>
+        <v>30.533096949259328</v>
       </c>
       <c r="E109">
         <v>5.7844444444444445</v>
       </c>
       <c r="F109">
-        <v>5.067836744747796</v>
+        <v>5.056587302123366</v>
       </c>
       <c r="G109" s="2">
-        <v>1.6435047812917616</v>
+        <v>1.6199720620847442</v>
       </c>
       <c r="H109" t="inlineStr">
         <is>
@@ -8622,22 +8622,22 @@
         </is>
       </c>
       <c r="J109">
-        <v>-23.979279200236004</v>
+        <v>-24.301781336466668</v>
       </c>
       <c r="K109">
-        <v>6.120556195577</v>
+        <v>6.120554288228666</v>
       </c>
       <c r="L109">
-        <v>120.61365763346366</v>
+        <v>120.557861328125</v>
       </c>
       <c r="M109">
         <v>5.7844444444444445</v>
       </c>
       <c r="N109">
-        <v>5.067898776532083</v>
+        <v>5.056648711509736</v>
       </c>
       <c r="O109" s="2">
-        <v>1.165479653972875</v>
+        <v>1.162364311401517</v>
       </c>
       <c r="P109" t="inlineStr">
         <is>
@@ -8652,22 +8652,22 @@
         </is>
       </c>
       <c r="B110">
-        <v>-73.70960744222</v>
+        <v>-74.34720357259134</v>
       </c>
       <c r="C110">
-        <v>18.59992535909</v>
+        <v>18.599923451741667</v>
       </c>
       <c r="D110">
-        <v>30.623664855957</v>
+        <v>30.613504409790004</v>
       </c>
       <c r="E110">
         <v>5.7844444444444445</v>
       </c>
       <c r="F110">
-        <v>5.058254389088974</v>
+        <v>5.051088601320718</v>
       </c>
       <c r="G110" s="2">
-        <v>1.6228198205899151</v>
+        <v>1.6078257237738784</v>
       </c>
       <c r="H110" t="inlineStr">
         <is>
@@ -8680,22 +8680,22 @@
         </is>
       </c>
       <c r="J110">
-        <v>-24.252825419108</v>
+        <v>-24.462598164876667</v>
       </c>
       <c r="K110">
-        <v>6.119661966959667</v>
+        <v>6.1196630795796665</v>
       </c>
       <c r="L110">
-        <v>120.91321818033866</v>
+        <v>120.87309773763033</v>
       </c>
       <c r="M110">
         <v>5.7844444444444445</v>
       </c>
       <c r="N110">
-        <v>5.058211984117502</v>
+        <v>5.051047483500603</v>
       </c>
       <c r="O110" s="2">
-        <v>1.157621370953317</v>
+        <v>1.1556788098364836</v>
       </c>
       <c r="P110" t="inlineStr">
         <is>
@@ -8710,22 +8710,22 @@
         </is>
       </c>
       <c r="B111">
-        <v>-73.52435302734366</v>
+        <v>-74.10671742757168</v>
       </c>
       <c r="C111">
-        <v>18.599953969319667</v>
+        <v>18.599953333537</v>
       </c>
       <c r="D111">
-        <v>30.630510965983333</v>
+        <v>30.624097188313666</v>
       </c>
       <c r="E111">
         <v>5.7844444444444445</v>
       </c>
       <c r="F111">
-        <v>5.060364851750048</v>
+        <v>5.053775805161672</v>
       </c>
       <c r="G111" s="2">
-        <v>1.6272001490397003</v>
+        <v>1.613399088217573</v>
       </c>
       <c r="H111" t="inlineStr">
         <is>
@@ -8738,22 +8738,22 @@
         </is>
       </c>
       <c r="J111">
-        <v>-24.191566467285</v>
+        <v>-24.383182525635</v>
       </c>
       <c r="K111">
-        <v>6.119787534077999</v>
+        <v>6.119788010915</v>
       </c>
       <c r="L111">
-        <v>120.94047292073567</v>
+        <v>120.91515858968067</v>
       </c>
       <c r="M111">
         <v>5.7844444444444445</v>
       </c>
       <c r="N111">
-        <v>5.060348798839903</v>
+        <v>5.053759948278408</v>
       </c>
       <c r="O111" s="2">
-        <v>1.1579578772972323</v>
+        <v>1.1560130842732599</v>
       </c>
       <c r="P111" t="inlineStr">
         <is>
@@ -8768,22 +8768,22 @@
         </is>
       </c>
       <c r="B112">
-        <v>-73.28684488932299</v>
+        <v>-73.86626180013033</v>
       </c>
       <c r="C112">
-        <v>18.59997113545733</v>
+        <v>18.599972407023</v>
       </c>
       <c r="D112">
-        <v>30.629402796427335</v>
+        <v>30.622621536255</v>
       </c>
       <c r="E112">
         <v>5.7844444444444445</v>
       </c>
       <c r="F112">
-        <v>5.063087926043667</v>
+        <v>5.0564825656140435</v>
       </c>
       <c r="G112" s="2">
-        <v>1.6329250400736652</v>
+        <v>1.6190998471408604</v>
       </c>
       <c r="H112" t="inlineStr">
         <is>
@@ -8796,22 +8796,22 @@
         </is>
       </c>
       <c r="J112">
-        <v>-24.113525390625</v>
+        <v>-24.304182688395333</v>
       </c>
       <c r="K112">
-        <v>6.119892120361333</v>
+        <v>6.119893391927</v>
       </c>
       <c r="L112">
-        <v>120.936030069987</v>
+        <v>120.90924835205065</v>
       </c>
       <c r="M112">
         <v>5.7844444444444445</v>
       </c>
       <c r="N112">
-        <v>5.063081737824568</v>
+        <v>5.05647614256255</v>
       </c>
       <c r="O112" s="2">
-        <v>1.158973893804956</v>
+        <v>1.1570592508150843</v>
       </c>
       <c r="P112" t="inlineStr">
         <is>
@@ -8826,22 +8826,22 @@
         </is>
       </c>
       <c r="B113">
-        <v>-73.20691172281933</v>
+        <v>-73.79817199707</v>
       </c>
       <c r="C113">
-        <v>18.599981307983334</v>
+        <v>18.599981307983665</v>
       </c>
       <c r="D113">
-        <v>30.62872187296567</v>
+        <v>30.621356964111335</v>
       </c>
       <c r="E113">
         <v>5.7844444444444445</v>
       </c>
       <c r="F113">
-        <v>5.064009210726708</v>
+        <v>5.057252930087406</v>
       </c>
       <c r="G113" s="2">
-        <v>1.6348632070905662</v>
+        <v>1.6207277957734516</v>
       </c>
       <c r="H113" t="inlineStr">
         <is>
@@ -8854,22 +8854,22 @@
         </is>
       </c>
       <c r="J113">
-        <v>-24.087431589762332</v>
+        <v>-24.281985600789668</v>
       </c>
       <c r="K113">
-        <v>6.119934399922667</v>
+        <v>6.119934717814333</v>
       </c>
       <c r="L113">
-        <v>120.93350982666033</v>
+        <v>120.90442657470733</v>
       </c>
       <c r="M113">
         <v>5.7844444444444445</v>
       </c>
       <c r="N113">
-        <v>5.064001144124351</v>
+        <v>5.057244637132175</v>
       </c>
       <c r="O113" s="2">
-        <v>1.1593295940538657</v>
+        <v>1.1574009172606454</v>
       </c>
       <c r="P113" t="inlineStr">
         <is>
@@ -8884,22 +8884,22 @@
         </is>
       </c>
       <c r="B114">
-        <v>-73.57988484700533</v>
+        <v>-74.11598459879568</v>
       </c>
       <c r="C114">
-        <v>18.599974314371668</v>
+        <v>18.599973678589</v>
       </c>
       <c r="D114">
-        <v>30.63168334960934</v>
+        <v>30.625796000163003</v>
       </c>
       <c r="E114">
         <v>5.7844444444444445</v>
       </c>
       <c r="F114">
-        <v>5.0597322237473294</v>
+        <v>5.053672837177586</v>
       </c>
       <c r="G114" s="2">
-        <v>1.6258608926548508</v>
+        <v>1.6131683742099063</v>
       </c>
       <c r="H114" t="inlineStr">
         <is>
@@ -8912,22 +8912,22 @@
         </is>
       </c>
       <c r="J114">
-        <v>-24.21028010050467</v>
+        <v>-24.386686325073327</v>
       </c>
       <c r="K114">
-        <v>6.119886398315334</v>
+        <v>6.119884808858</v>
       </c>
       <c r="L114">
-        <v>120.94559733072934</v>
+        <v>120.92235056559267</v>
       </c>
       <c r="M114">
         <v>5.7844444444444445</v>
       </c>
       <c r="N114">
-        <v>5.059713502597948</v>
+        <v>5.053653726908456</v>
       </c>
       <c r="O114" s="2">
-        <v>1.157654570941569</v>
+        <v>1.1558639826643111</v>
       </c>
       <c r="P114" t="inlineStr">
         <is>
@@ -8942,22 +8942,22 @@
         </is>
       </c>
       <c r="B115">
-        <v>-76.26045481363934</v>
+        <v>-76.29179382324233</v>
       </c>
       <c r="C115">
-        <v>18.599990208943666</v>
+        <v>18.599988937377997</v>
       </c>
       <c r="D115">
-        <v>30.715451558431003</v>
+        <v>30.714287439981998</v>
       </c>
       <c r="E115">
         <v>5.7844444444444445</v>
       </c>
       <c r="F115">
-        <v>5.030422762887383</v>
+        <v>5.030094154526985</v>
       </c>
       <c r="G115" s="2">
-        <v>1.5635343359839362</v>
+        <v>1.5628487411623977</v>
       </c>
       <c r="H115" t="inlineStr">
         <is>
@@ -8970,22 +8970,22 @@
         </is>
       </c>
       <c r="J115">
-        <v>-25.092327117920004</v>
+        <v>-25.102639516194667</v>
       </c>
       <c r="K115">
-        <v>6.119988282521667</v>
+        <v>6.119984785715666</v>
       </c>
       <c r="L115">
-        <v>121.27658589680968</v>
+        <v>121.27198537190765</v>
       </c>
       <c r="M115">
         <v>5.7844444444444445</v>
       </c>
       <c r="N115">
-        <v>5.030415995174932</v>
+        <v>5.030086963502034</v>
       </c>
       <c r="O115" s="2">
-        <v>1.1421940410406406</v>
+        <v>1.1421394027571534</v>
       </c>
       <c r="P115" t="inlineStr">
         <is>
@@ -9000,22 +9000,22 @@
         </is>
       </c>
       <c r="B116">
-        <v>-77.95453898112001</v>
+        <v>-77.93149820963534</v>
       </c>
       <c r="C116">
-        <v>18.599998474121335</v>
+        <v>18.599995930989333</v>
       </c>
       <c r="D116">
-        <v>30.72404607137033</v>
+        <v>30.724409739176334</v>
       </c>
       <c r="E116">
         <v>5.7844444444444445</v>
       </c>
       <c r="F116">
-        <v>5.013100122942445</v>
+        <v>5.013329786558203</v>
       </c>
       <c r="G116" s="2">
-        <v>1.5268435644098386</v>
+        <v>1.5273278199865759</v>
       </c>
       <c r="H116" t="inlineStr">
         <is>
@@ -9028,22 +9028,22 @@
         </is>
       </c>
       <c r="J116">
-        <v>-25.649628321330002</v>
+        <v>-25.642045338948666</v>
       </c>
       <c r="K116">
-        <v>6.120010058085</v>
+        <v>6.120006084442</v>
       </c>
       <c r="L116">
-        <v>121.31058502197233</v>
+        <v>121.31202189127565</v>
       </c>
       <c r="M116">
         <v>5.7844444444444445</v>
       </c>
       <c r="N116">
-        <v>5.0130993329234075</v>
+        <v>5.01332865246826</v>
       </c>
       <c r="O116" s="2">
-        <v>1.1351551085217864</v>
+        <v>1.1352228435926774</v>
       </c>
       <c r="P116" t="inlineStr">
         <is>
@@ -9058,22 +9058,22 @@
         </is>
       </c>
       <c r="B117">
-        <v>-61.526178995768326</v>
+        <v>-61.51789983113599</v>
       </c>
       <c r="C117">
         <v>18.59997113545733</v>
       </c>
       <c r="D117">
-        <v>30.864473978678337</v>
+        <v>30.86422602335633</v>
       </c>
       <c r="E117">
         <v>5.7844444444444445</v>
       </c>
       <c r="F117">
-        <v>5.229560967596806</v>
+        <v>5.2297051740787115</v>
       </c>
       <c r="G117" s="2">
-        <v>1.9741861020171456</v>
+        <v>1.9744811782477505</v>
       </c>
       <c r="H117" t="inlineStr">
         <is>
@@ -9086,22 +9086,22 @@
         </is>
       </c>
       <c r="J117">
-        <v>-20.243912378946998</v>
+        <v>-20.241183598836333</v>
       </c>
       <c r="K117">
-        <v>6.119933287302667</v>
+        <v>6.1199248631793335</v>
       </c>
       <c r="L117">
-        <v>121.86480458577499</v>
+        <v>121.86382548014333</v>
       </c>
       <c r="M117">
         <v>5.7844444444444445</v>
       </c>
       <c r="N117">
-        <v>5.229560754058314</v>
+        <v>5.229703733774843</v>
       </c>
       <c r="O117" s="2">
-        <v>1.1930356296666178</v>
+        <v>1.1930864414103188</v>
       </c>
       <c r="P117" t="inlineStr">
         <is>
@@ -9526,13 +9526,13 @@
         </is>
       </c>
       <c r="B123">
-        <v>-66.2182411876153</v>
+        <v>-66.49143462075558</v>
       </c>
       <c r="C123">
-        <v>387.59333725408175</v>
+        <v>362.8155234661407</v>
       </c>
       <c r="D123" s="2">
-        <v>1.1440261897414763</v>
+        <v>1.7246582691226988</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -9545,13 +9545,13 @@
         </is>
       </c>
       <c r="G123">
-        <v>-21.787659152736435</v>
+        <v>-21.87755140848512</v>
       </c>
       <c r="H123">
-        <v>387.59333725408175</v>
+        <v>362.8155234661407</v>
       </c>
       <c r="I123" s="2">
-        <v>3.4769867486078736</v>
+        <v>5.241674463625814</v>
       </c>
       <c r="J123" t="inlineStr">
         <is>
@@ -9596,13 +9596,13 @@
         </is>
       </c>
       <c r="B124">
-        <v>-72.92718797389094</v>
+        <v>-73.16358277398334</v>
       </c>
       <c r="C124">
-        <v>387.59333725408175</v>
+        <v>362.8155234661407</v>
       </c>
       <c r="D124" s="2">
-        <v>1.0387813415261704</v>
+        <v>1.5673781708964556</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -9615,13 +9615,13 @@
         </is>
       </c>
       <c r="G124">
-        <v>-23.995632429433044</v>
+        <v>-24.073413799738255</v>
       </c>
       <c r="H124">
-        <v>387.59333725408175</v>
+        <v>362.8155234661407</v>
       </c>
       <c r="I124" s="2">
-        <v>3.157049616426365</v>
+        <v>4.763553831561865</v>
       </c>
       <c r="J124" t="inlineStr">
         <is>
@@ -9666,13 +9666,13 @@
         </is>
       </c>
       <c r="B125">
-        <v>-73.1681154413481</v>
+        <v>-73.57489603915427</v>
       </c>
       <c r="C125">
         <v>491.79</v>
       </c>
       <c r="D125" s="3">
-        <v>0.918952064142182</v>
+        <v>0.9138713655597739</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -9685,13 +9685,13 @@
         </is>
       </c>
       <c r="G125">
-        <v>-24.074543884354515</v>
+        <v>-24.20838321233366</v>
       </c>
       <c r="H125">
         <v>491.79</v>
       </c>
       <c r="I125" s="2">
-        <v>2.792908187054655</v>
+        <v>2.7774672155703466</v>
       </c>
       <c r="J125" t="inlineStr">
         <is>
@@ -9736,13 +9736,13 @@
         </is>
       </c>
       <c r="B126">
-        <v>-72.747284230178</v>
+        <v>-72.80487964039108</v>
       </c>
       <c r="C126">
-        <v>387.59333725408175</v>
+        <v>362.8155234661407</v>
       </c>
       <c r="D126" s="2">
-        <v>1.0413502436400748</v>
+        <v>1.5751005030286103</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -9755,13 +9755,13 @@
         </is>
       </c>
       <c r="G126">
-        <v>-23.93611706756957</v>
+        <v>-23.95506459933124</v>
       </c>
       <c r="H126">
-        <v>387.59333725408175</v>
+        <v>362.8155234661407</v>
       </c>
       <c r="I126" s="2">
-        <v>3.1648993837805333</v>
+        <v>4.787088010930216</v>
       </c>
       <c r="J126" t="inlineStr">
         <is>
@@ -9806,13 +9806,13 @@
         </is>
       </c>
       <c r="B127">
-        <v>-72.8618375583078</v>
+        <v>-73.26930388395937</v>
       </c>
       <c r="C127">
         <v>491.79</v>
       </c>
       <c r="D127" s="3">
-        <v>0.9228149188580784</v>
+        <v>0.9176829470184241</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -9825,13 +9825,13 @@
         </is>
       </c>
       <c r="G127">
-        <v>-23.973925351032513</v>
+        <v>-24.107997530643726</v>
       </c>
       <c r="H127">
         <v>491.79</v>
       </c>
       <c r="I127" s="2">
-        <v>2.804630019060457</v>
+        <v>2.789032586748607</v>
       </c>
       <c r="J127" t="inlineStr">
         <is>
@@ -9876,13 +9876,13 @@
         </is>
       </c>
       <c r="B128">
-        <v>-72.6994006691911</v>
+        <v>-72.75102589948524</v>
       </c>
       <c r="C128">
-        <v>387.59333725408175</v>
+        <v>362.8155234661407</v>
       </c>
       <c r="D128" s="2">
-        <v>1.0420361304209982</v>
+        <v>1.5762664667156097</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -9895,13 +9895,13 @@
         </is>
       </c>
       <c r="G128">
-        <v>-23.920534804584495</v>
+        <v>-23.937519071634018</v>
       </c>
       <c r="H128">
-        <v>387.59333725408175</v>
+        <v>362.8155234661407</v>
       </c>
       <c r="I128" s="2">
-        <v>3.1669610556838683</v>
+        <v>4.790596811697474</v>
       </c>
       <c r="J128" t="inlineStr">
         <is>
@@ -9946,13 +9946,13 @@
         </is>
       </c>
       <c r="B129">
-        <v>-74.2133416088431</v>
+        <v>-74.41161868910268</v>
       </c>
       <c r="C129">
         <v>491.79</v>
       </c>
       <c r="D129" s="3">
-        <v>0.9060094756090107</v>
+        <v>0.9035953242079797</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -9965,13 +9965,13 @@
         </is>
       </c>
       <c r="G129">
-        <v>-24.418644099885476</v>
+        <v>-24.483886199761958</v>
       </c>
       <c r="H129">
         <v>491.79</v>
       </c>
       <c r="I129" s="2">
-        <v>2.7535513617865317</v>
+        <v>2.746213986032741</v>
       </c>
       <c r="J129" t="inlineStr">
         <is>
@@ -10016,13 +10016,13 @@
         </is>
       </c>
       <c r="B130">
-        <v>-76.23322758967643</v>
+        <v>-76.23844296081845</v>
       </c>
       <c r="C130">
         <v>491.79</v>
       </c>
       <c r="D130" s="3">
-        <v>0.8820037251489234</v>
+        <v>0.8819433884395594</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -10035,13 +10035,13 @@
         </is>
       </c>
       <c r="G130">
-        <v>-25.08319830763531</v>
+        <v>-25.08491431222198</v>
       </c>
       <c r="H130">
         <v>491.79</v>
       </c>
       <c r="I130" s="2">
-        <v>2.6805987772999864</v>
+        <v>2.6804154033510224</v>
       </c>
       <c r="J130" t="inlineStr">
         <is>
@@ -10086,13 +10086,13 @@
         </is>
       </c>
       <c r="B131">
-        <v>-68.90772643942142</v>
+        <v>-68.89444833091554</v>
       </c>
       <c r="C131">
         <v>491.79</v>
       </c>
       <c r="D131" s="3">
-        <v>0.9757685268187011</v>
+        <v>0.9759565878408824</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -10105,13 +10105,13 @@
         </is>
       </c>
       <c r="G131">
-        <v>-22.67279015592485</v>
+        <v>-22.66841855762845</v>
       </c>
       <c r="H131">
         <v>491.79</v>
       </c>
       <c r="I131" s="2">
-        <v>2.9655807799486764</v>
+        <v>2.9661526913880443</v>
       </c>
       <c r="J131" t="inlineStr">
         <is>
@@ -10484,16 +10484,16 @@
         </is>
       </c>
       <c r="B136">
-        <v>82841.66183943089</v>
+        <v>124656.32338853959</v>
       </c>
       <c r="C136">
-        <v>7.946163259608169</v>
+        <v>9.77653724016467</v>
       </c>
       <c r="D136">
-        <v>75.50813900966672</v>
+        <v>61.371422750279834</v>
       </c>
       <c r="E136">
-        <v>57.81932890503286</v>
+        <v>59.76105665571706</v>
       </c>
       <c r="F136" t="inlineStr">
         <is>
@@ -10558,16 +10558,16 @@
         </is>
       </c>
       <c r="B137">
-        <v>82841.66183943089</v>
+        <v>124656.32338853959</v>
       </c>
       <c r="C137">
-        <v>7.946163259608169</v>
+        <v>9.77653724016467</v>
       </c>
       <c r="D137">
-        <v>75.50813900966672</v>
+        <v>61.371422750279834</v>
       </c>
       <c r="E137">
-        <v>57.81932890503286</v>
+        <v>59.76105665571706</v>
       </c>
       <c r="F137" t="inlineStr">
         <is>
@@ -10706,16 +10706,16 @@
         </is>
       </c>
       <c r="B139">
-        <v>82841.66183943089</v>
+        <v>124656.32338853959</v>
       </c>
       <c r="C139">
-        <v>7.946163259608169</v>
+        <v>9.77653724016467</v>
       </c>
       <c r="D139">
-        <v>75.50813900966672</v>
+        <v>61.371422750279834</v>
       </c>
       <c r="E139">
-        <v>57.81932890503286</v>
+        <v>59.76105665571706</v>
       </c>
       <c r="F139" t="inlineStr">
         <is>
@@ -10854,16 +10854,16 @@
         </is>
       </c>
       <c r="B141">
-        <v>82841.66183943089</v>
+        <v>124656.32338853959</v>
       </c>
       <c r="C141">
-        <v>7.946163259608169</v>
+        <v>9.77653724016467</v>
       </c>
       <c r="D141">
-        <v>75.50813900966672</v>
+        <v>61.371422750279834</v>
       </c>
       <c r="E141">
-        <v>57.81932890503286</v>
+        <v>59.76105665571706</v>
       </c>
       <c r="F141" t="inlineStr">
         <is>
@@ -11314,7 +11314,7 @@
         </is>
       </c>
       <c r="B147" s="2">
-        <v>1.657138996173068</v>
+        <v>1.657175741031117</v>
       </c>
       <c r="C147" t="inlineStr">
         <is>
@@ -11394,7 +11394,7 @@
         </is>
       </c>
       <c r="B148" s="2">
-        <v>1.1351551085217864</v>
+        <v>1.1352228435926774</v>
       </c>
       <c r="C148" t="inlineStr">
         <is>
@@ -11474,7 +11474,7 @@
         </is>
       </c>
       <c r="B149" s="3">
-        <v>0.8820037251489234</v>
+        <v>0.8819433884395594</v>
       </c>
       <c r="C149" t="inlineStr">
         <is>
@@ -11554,7 +11554,7 @@
         </is>
       </c>
       <c r="B150" s="3">
-        <v>0.8820037251489234</v>
+        <v>0.8819433884395594</v>
       </c>
       <c r="C150" t="inlineStr">
         <is>
@@ -11798,7 +11798,7 @@
         </is>
       </c>
       <c r="B153">
-        <v>20.189088</v>
+        <v>20.138544</v>
       </c>
       <c r="C153" t="inlineStr">
         <is>

</xml_diff>